<commit_message>
Add cards-promo, carousel-quote, isi blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/cards-promo/cards-promo.css
- blocks/carousel-quote/carousel-quote.css
- blocks/isi/README.md
- blocks/isi/isi.css
- blocks/isi/isi.js
- blocks/isi/metadata.json
- tools/importer/import-how-vyepti-works.bundle.js
- tools/importer/import-how-vyepti-works.js
- tools/importer/page-templates.json
- tools/importer/parsers/isi.js
- tools/importer/reports/how-vyepti-works.report.json
- tools/importer/reports/import-how-vyepti-works.report.xlsx
- tools/importer/transformers/vyepti-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-how-vyepti-works.report.xlsx
+++ b/tools/importer/reports/import-how-vyepti-works.report.xlsx
@@ -40,7 +40,7 @@
     <t>how-vyepti-works.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-feature","columns-media","columns-cta","carousel-quote","cards-promo"]</t>
+    <t>["hero-banner","cards-feature","columns-media","columns-cta","carousel-quote","cards-promo","isi"]</t>
   </si>
   <si>
     <t>how-vyepti-works</t>
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-09-16T12:43:39.329Z</t>
+    <t>2026-09-16T13:56:27.554Z</t>
   </si>
   <si>
     <t>How VYEPTI® Works: Designed to Help Prevent Migraine Attacks</t>

</xml_diff>